<commit_message>
Add word "besluttede" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -311,9 +311,95 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>42dc3954-91f0-4b4c-bcbf-5d892975a793</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C2" t="str">
+        <v>besluttede</v>
+      </c>
+      <c r="D2" t="str">
+        <v>beslutte</v>
+      </c>
+      <c r="E2" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[beˈsludə]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004277_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>endeligt aftale eller afgøre noget som man har været i tvivl eller uenige om, fx på baggrund af en diskussion, en overvejelse el.lign.</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Decided</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Hannah Berlin, 1939 Jeg var knap tolv år gammel, da jeg besluttede mig for at slå mine forældre ihjel.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -322,28 +408,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -425,8 +511,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "ihjel" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -397,9 +397,95 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>04975e11-6b0f-40ac-af74-22fdc9996b2b</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ihjel</v>
+      </c>
+      <c r="D3" t="str">
+        <v>ihjel</v>
+      </c>
+      <c r="E3" t="str">
+        <v>adverbium</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>[iˈjεl]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/11022/11022871_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v>til døden indtræffer; med døden til følge</v>
+      </c>
+      <c r="K3" t="str">
+        <v>to death</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Hannah Berlin, 1939 Jeg var knap tolv år gammel, da jeg besluttede mig for at slå mine forældre ihjel.</v>
+      </c>
+      <c r="M3" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "tunge" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -483,9 +483,95 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fe218f48-5066-4c08-b911-bd4e99eefec0</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C4" t="str">
+        <v>tunge</v>
+      </c>
+      <c r="D4" t="str">
+        <v>tunge</v>
+      </c>
+      <c r="E4" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F4" t="str">
+        <v>en</v>
+      </c>
+      <c r="G4" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[ˈtɔŋə]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002852_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>muskelfyldt, aflangt og bevægeligt organ i mundhulen som bruges til at smage, slikke og (hos mennesket) frembringe tale med</v>
+      </c>
+      <c r="K4" t="str">
+        <v>tongue</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Jeg vidste altid hvornår, for papa lukkede de store tunge dobbeltvinduer og trak de tykke grønlige bronzefarvede gardiner for.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O4" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "grønlige" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -569,9 +569,95 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>f54fa6ee-5adf-41ca-a63c-5f0917fff715</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C5" t="str">
+        <v>grønlige</v>
+      </c>
+      <c r="D5" t="str">
+        <v>grønlig</v>
+      </c>
+      <c r="E5" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[ˈgʁɶnli]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/11018/11018975_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>med en antydning af grøn farve; med et grønt skær</v>
+      </c>
+      <c r="K5" t="str">
+        <v>greenish</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Jeg vidste altid hvornår, for papa lukkede de store tunge dobbeltvinduer og trak de tykke grønlige bronzefarvede gardiner for.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O5" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "dampende" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -655,9 +655,95 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>8cea12a4-108f-4fc6-b9c0-4be20acb5036</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C6" t="str">
+        <v>dampende</v>
+      </c>
+      <c r="D6" t="str">
+        <v>dampe</v>
+      </c>
+      <c r="E6" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H6" t="str">
+        <v>[ˈdɑmbə]</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/11008/11008323_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v>udsende damp eller røg</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Steaming</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Så sagde han det samme, som han sagde hver aften efter aftensmaden, som på det tidspunkt ikke var meget andet end en dampende portion suppe uden smag.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O6" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "knækkede" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -741,9 +741,95 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>7b0055c0-6fc7-45bd-9921-d98f4e3b16e7</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C7" t="str">
+        <v>knækkede</v>
+      </c>
+      <c r="D7" t="str">
+        <v>knække</v>
+      </c>
+      <c r="E7" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>-r, -de (eller uofficiel form: knak), -t Se bøjning i skema</v>
+      </c>
+      <c r="H7" t="str">
+        <v>[ˈknεgə]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11026/11026736_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>pludselig briste eller gå i to eller flere stykker som følge af et stærkt tryk, ofte ledsaget af en kort, skarp lyd</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Broke</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Vi må rejse.” Så begyndte mama altid at råbe op, hendes stemme knækkede over, mens hun bebrejdede ham alt.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v/>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bebrejdede" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -827,9 +827,95 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>33d1b4ab-8bea-42cb-bdeb-cb62fa2ae2b7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C8" t="str">
+        <v>bebrejdede</v>
+      </c>
+      <c r="D8" t="str">
+        <v>bebrejde</v>
+      </c>
+      <c r="E8" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H8" t="str">
+        <v>[beˈbʁɑjˀdə]</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003699_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v>udtrykke utilfredshed med noget som nogen gør, tænker, føler el.lign.</v>
+      </c>
+      <c r="K8" t="str">
+        <v>blamed</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Vi må rejse.” Så begyndte mama altid at råbe op, hendes stemme knækkede over, mens hun bebrejdede ham alt.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O8" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "travede" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -913,9 +913,95 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>e2cbefd7-f4e1-4e96-b3de-3094711c2af7</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C9" t="str">
+        <v>travede</v>
+      </c>
+      <c r="D9" t="str">
+        <v>trave</v>
+      </c>
+      <c r="E9" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H9" t="str">
+        <v>[ˈtʁɑːvə]</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002172_1.mp3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>gå rask og vedholdende over en længere strækning</v>
+      </c>
+      <c r="K9" t="str">
+        <v>trotted</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Hun travede rundt i hele lejligheden – hendes lillebitte fort i hjertet af en druknende by; det eneste sted, hun havde opholdt sig de sidste fire måneder – indtil hun havde kørt sig selv træt.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N9" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O9" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "fort" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AB10"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -999,9 +999,95 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>d21b108e-003e-481a-8171-08f10cead75b</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C10" t="str">
+        <v>fort</v>
+      </c>
+      <c r="D10" t="str">
+        <v>fort</v>
+      </c>
+      <c r="E10" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F10" t="str">
+        <v>et</v>
+      </c>
+      <c r="G10" t="str">
+        <v>-et, -er, -erne</v>
+      </c>
+      <c r="H10" t="str">
+        <v>[ˈfɒːd]</v>
+      </c>
+      <c r="I10" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015314_1.mp3</v>
+      </c>
+      <c r="J10" t="str">
+        <v>befæstet (og bemandet) militæranlæg der er placeret ud fra strategiske hensyn, fx ved en havn ofte om historiske forhold</v>
+      </c>
+      <c r="K10" t="str">
+        <v>fortress</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Hun travede rundt i hele lejligheden – hendes lillebitte fort i hjertet af en druknende by; det eneste sted, hun havde opholdt sig de sidste fire måneder – indtil hun havde kørt sig selv træt.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N10" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O10" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "eneste" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1085,9 +1085,95 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>d4e4fb0e-8d4a-4d93-b595-2c9032a47447</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C11" t="str">
+        <v>eneste</v>
+      </c>
+      <c r="D11" t="str">
+        <v>eneste</v>
+      </c>
+      <c r="E11" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>-, -</v>
+      </c>
+      <c r="H11" t="str">
+        <v>[ˈeːnəsdə]</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://static.ordnet.dk/mp3/11011/11011387_1.mp3</v>
+      </c>
+      <c r="J11" t="str">
+        <v>som der kun er én eller ét af; som udgør hele den forholdsvis lille mængde eller det forholdsvis lille antal af en given slags</v>
+      </c>
+      <c r="K11" t="str">
+        <v>only</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Hun travede rundt i hele lejligheden – hendes lillebitte fort i hjertet af en druknende by; det eneste sted, hun havde opholdt sig de sidste fire måneder – indtil hun havde kørt sig selv træt.</v>
+      </c>
+      <c r="M11" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N11" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O11" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "træt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1171,9 +1171,95 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>0f1c36fe-9aa1-4440-8e86-78bbcee8efbe</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C12" t="str">
+        <v>træt</v>
+      </c>
+      <c r="D12" t="str">
+        <v>træt</v>
+      </c>
+      <c r="E12" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v>-, -te -tere, -test</v>
+      </c>
+      <c r="H12" t="str">
+        <v>[ˈtʁad]</v>
+      </c>
+      <c r="I12" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002730_1.mp3</v>
+      </c>
+      <c r="J12" t="str">
+        <v>slap, udmattet eller uden energi pga. fx anstrengelse eller mangel på hvile; som føler trang til at sove eller hvile sig</v>
+      </c>
+      <c r="K12" t="str">
+        <v>tired</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Hun travede rundt i hele lejligheden – hendes lillebitte fort i hjertet af en druknende by; det eneste sted, hun havde opholdt sig de sidste fire måneder – indtil hun havde kørt sig selv træt.</v>
+      </c>
+      <c r="M12" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N12" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O12" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "slog" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1257,9 +1257,95 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>11137a32-58b8-4f70-882d-d42bbdecf341</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C13" t="str">
+        <v>slog</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>-r, slog, -et</v>
+      </c>
+      <c r="H13" t="str">
+        <v>[ˈslɔˀ]</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047901_1.mp3</v>
+      </c>
+      <c r="J13" t="str">
+        <v>bevæge hånden eller et redskab (flere gange) hurtigt mod noget så det bliver ramt fx for at bearbejde eller ødelægge noget, for at drive en pæl eller et søm ind eller ned i noget, eller for at påføre nogen smerte</v>
+      </c>
+      <c r="K13" t="str">
+        <v>beat</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Så slog hun armene om papa, og hendes kraftesløse støn ophørte langt om længe.</v>
+      </c>
+      <c r="M13" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N13" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O13" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "armene" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1343,9 +1343,95 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>7d56c339-15ff-4c02-82bf-d85bc52427fd</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C14" t="str">
+        <v>armene</v>
+      </c>
+      <c r="D14" t="str">
+        <v>arm</v>
+      </c>
+      <c r="E14" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F14" t="str">
+        <v>en</v>
+      </c>
+      <c r="G14" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H14" t="str">
+        <v>[ˈɑˀm]</v>
+      </c>
+      <c r="I14" t="str">
+        <v>https://static.ordnet.dk/mp3/11002/11002463_1.mp3</v>
+      </c>
+      <c r="J14" t="str">
+        <v>hvert af de to symmetriske lemmer der udgår fra overkroppen på mennesker, især stykket mellem skulder og håndled eller tilsvarende lem hos andre dyr der går på to ben</v>
+      </c>
+      <c r="K14" t="str">
+        <v>The arms</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Så slog hun armene om papa, og hendes kraftesløse støn ophørte langt om længe.</v>
+      </c>
+      <c r="M14" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N14" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O14" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kraftesløse" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1429,9 +1429,95 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ce4cfdb0-c250-42e6-91b1-a1c05f1722cf</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C15" t="str">
+        <v>kraftesløse</v>
+      </c>
+      <c r="D15" t="str">
+        <v>kraftesløs</v>
+      </c>
+      <c r="E15" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H15" t="str">
+        <v>[ˈkʁɑfdəs-]</v>
+      </c>
+      <c r="I15" t="str">
+        <v>https://static.ordnet.dk/mp3/11027/11027874_1.mp3</v>
+      </c>
+      <c r="J15" t="str">
+        <v>udmattet, energiforladt og uden styrke, fx pga. sygdom eller anstrengelse</v>
+      </c>
+      <c r="K15" t="str">
+        <v>powerless</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Så slog hun armene om papa, og hendes kraftesløse støn ophørte langt om længe.</v>
+      </c>
+      <c r="M15" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N15" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O15" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "støn" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AB16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1515,9 +1515,95 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>ecdc8711-5c83-4964-85e7-997b838d32ae</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C16" t="str">
+        <v>støn</v>
+      </c>
+      <c r="D16" t="str">
+        <v>støn</v>
+      </c>
+      <c r="E16" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F16" t="str">
+        <v>et</v>
+      </c>
+      <c r="G16" t="str">
+        <v>-net, -, -nene</v>
+      </c>
+      <c r="H16" t="str">
+        <v>[ˈsdœnˀ]</v>
+      </c>
+      <c r="I16" t="str">
+        <v>https://static.ordnet.dk/mp3/11051/11051161_1.mp3</v>
+      </c>
+      <c r="J16" t="str">
+        <v>højlydt, besværet udånding forårsaget af smerte, vellyst eller hård fysisk anstrengelse</v>
+      </c>
+      <c r="K16" t="str">
+        <v>groan</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Så slog hun armene om papa, og hendes kraftesløse støn ophørte langt om længe.</v>
+      </c>
+      <c r="M16" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N16" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O16" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ophørte" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1601,9 +1601,95 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>aa362b68-4a15-4759-9585-29e0622e85b1</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C17" t="str">
+        <v>ophørte</v>
+      </c>
+      <c r="D17" t="str">
+        <v>ophøre</v>
+      </c>
+      <c r="E17" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v>-r, ophørte, ophørt</v>
+      </c>
+      <c r="H17" t="str">
+        <v>[ˈʌbˌhøˀʌ]</v>
+      </c>
+      <c r="I17" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037484_1.mp3</v>
+      </c>
+      <c r="J17" t="str">
+        <v>ikke blive ved længere; holde op</v>
+      </c>
+      <c r="K17" t="str">
+        <v>ceased</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Så slog hun armene om papa, og hendes kraftesløse støn ophørte langt om længe.</v>
+      </c>
+      <c r="M17" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N17" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O17" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v/>
+      </c>
+      <c r="AA17" t="str">
+        <v/>
+      </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "slog" in Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB17"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1289,7 +1289,7 @@
         <v>bevæge hånden eller et redskab (flere gange) hurtigt mod noget så det bliver ramt fx for at bearbejde eller ødelægge noget, for at drive en pæl eller et søm ind eller ned i noget, eller for at påføre nogen smerte</v>
       </c>
       <c r="K13" t="str">
-        <v>beat</v>
+        <v>wrap(arms around)/beat</v>
       </c>
       <c r="L13" t="str">
         <v>Så slog hun armene om papa, og hendes kraftesløse støn ophørte langt om længe.</v>

</xml_diff>

<commit_message>
Add word "druknende" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB17"/>
+  <dimension ref="A1:AB18"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1687,9 +1687,95 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>10ff1ecb-d0af-438d-b61c-f6c5ee25b1b1</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C18" t="str">
+        <v>druknende</v>
+      </c>
+      <c r="D18" t="str">
+        <v>drukne</v>
+      </c>
+      <c r="E18" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H18" t="str">
+        <v>[ˈdʁɔgnə]</v>
+      </c>
+      <c r="I18" t="str">
+        <v>https://static.ordnet.dk/mp3/11009/11009790_1.mp3</v>
+      </c>
+      <c r="J18" t="str">
+        <v>dø af iltmangel fordi man har hovedet under vand (eller en anden væske) og ikke kan trække vejret</v>
+      </c>
+      <c r="K18" t="str">
+        <v>drowning</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Hun travede rundt i hele lejligheden – hendes lillebitte fort i hjertet af en druknende by; det eneste sted, hun havde opholdt sig de sidste fire måneder – indtil hun havde kørt sig selv træt.</v>
+      </c>
+      <c r="M18" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N18" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O18" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
+      <c r="AA18" t="str">
+        <v/>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "opholdt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB18"/>
+  <dimension ref="A1:AB19"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1773,9 +1773,95 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>0c228677-3ffe-4697-96c4-946ee07fecfd</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C19" t="str">
+        <v>opholdt</v>
+      </c>
+      <c r="D19" t="str">
+        <v>opholde</v>
+      </c>
+      <c r="E19" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v>-r, opholdt, opholdt</v>
+      </c>
+      <c r="H19" t="str">
+        <v>[ˈʌbˌhʌlˀə]</v>
+      </c>
+      <c r="I19" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037461_1.mp3</v>
+      </c>
+      <c r="J19" t="str">
+        <v>forårsage at nogen eller noget bliver afbrudt eller standset (og derfor ikke når noget planlagt i rette tid)</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Stayed</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Hun travede rundt i hele lejligheden – hendes lillebitte fort i hjertet af en druknende by; det eneste sted, hun havde opholdt sig de sidste fire måneder – indtil hun havde kørt sig selv træt.</v>
+      </c>
+      <c r="M19" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N19" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O19" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
+      </c>
+      <c r="AA19" t="str">
+        <v/>
+      </c>
+      <c r="AB19" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "modstand" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AB20"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1859,9 +1859,95 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>5672f5db-2048-42fb-984e-318de56f558e</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C20" t="str">
+        <v>modstand</v>
+      </c>
+      <c r="D20" t="str">
+        <v>modstand</v>
+      </c>
+      <c r="E20" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F20" t="str">
+        <v>en</v>
+      </c>
+      <c r="G20" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H20" t="str">
+        <v>[ˈmoðˌsdanˀ]</v>
+      </c>
+      <c r="I20" t="str">
+        <v>https://static.ordnet.dk/mp3/11034/11034125_1.mp3</v>
+      </c>
+      <c r="J20" t="str">
+        <v>forsøg på at modvirke en fysisk eller psykisk påvirkning med magt</v>
+      </c>
+      <c r="K20" t="str">
+        <v>resistance</v>
+      </c>
+      <c r="L20" t="str">
+        <v>De ville ikke gøre modstand.</v>
+      </c>
+      <c r="M20" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N20" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O20" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
+      <c r="AA20" t="str">
+        <v/>
+      </c>
+      <c r="AB20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "give slip" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB20"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1954,30 +1954,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2048,9 +2048,77 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>60f6f3ae-a546-4415-b33c-2c27bf67a29d</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C2" t="str">
+        <v>give slip</v>
+      </c>
+      <c r="D2" t="str">
+        <v>give=give · slip=Release</v>
+      </c>
+      <c r="E2" t="str">
+        <v>let go</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Jeg vidste, at papa allerede havde givet op og var klar til at give slip.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "sværere" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB20"/>
+  <dimension ref="A1:AB21"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1945,9 +1945,95 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>18e9d90c-bc69-4335-9172-63251bdfcf3c</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C21" t="str">
+        <v>sværere</v>
+      </c>
+      <c r="D21" t="str">
+        <v>svær</v>
+      </c>
+      <c r="E21" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H21" t="str">
+        <v>[ˈsvεˀɐ̯]</v>
+      </c>
+      <c r="I21" t="str">
+        <v>https://static.ordnet.dk/mp3/11051/11051804_1.mp3</v>
+      </c>
+      <c r="J21" t="str">
+        <v>som stiller særlig (fysisk eller psykisk) anstrengende krav for at kunne udføres; som volder besvær</v>
+      </c>
+      <c r="K21" t="str">
+        <v>harder</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Det ville være sværere med mama, men hun tog så mange sovepiller, at hun ville sove tungt, indhyllet i duften af sine jasmin- og geraniumparfumer.</v>
+      </c>
+      <c r="M21" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N21" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O21" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
+      </c>
+      <c r="Y21" t="str">
+        <v/>
+      </c>
+      <c r="Z21" t="str">
+        <v/>
+      </c>
+      <c r="AA21" t="str">
+        <v/>
+      </c>
+      <c r="AB21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1956,28 +2042,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "tungt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AB22"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2031,9 +2031,95 @@
         <v/>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>f7b300eb-fa18-41e2-a200-65ee6032a4ec</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C22" t="str">
+        <v>tungt</v>
+      </c>
+      <c r="D22" t="str">
+        <v>tung</v>
+      </c>
+      <c r="E22" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H22" t="str">
+        <v>[ˈtɔŋˀ]</v>
+      </c>
+      <c r="I22" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002851_1.mp3</v>
+      </c>
+      <c r="J22" t="str">
+        <v>som vejer meget; som er svær at løfte eller flytte</v>
+      </c>
+      <c r="K22" t="str">
+        <v>heavy</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Det ville være sværere med mama, men hun tog så mange sovepiller, at hun ville sove tungt, indhyllet i duften af sine jasmin- og geraniumparfumer.</v>
+      </c>
+      <c r="M22" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N22" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O22" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+      <c r="X22" t="str">
+        <v/>
+      </c>
+      <c r="Y22" t="str">
+        <v/>
+      </c>
+      <c r="Z22" t="str">
+        <v/>
+      </c>
+      <c r="AA22" t="str">
+        <v/>
+      </c>
+      <c r="AB22" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "indhyllet" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2117,9 +2117,95 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>a8c51c9d-78e8-4cec-9304-09ed03a09a7c</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C23" t="str">
+        <v>indhyllet</v>
+      </c>
+      <c r="D23" t="str">
+        <v>indhylle</v>
+      </c>
+      <c r="E23" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H23" t="str">
+        <v>[-ˌhylˀə]</v>
+      </c>
+      <c r="I23" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023327_1.mp3</v>
+      </c>
+      <c r="J23" t="str">
+        <v>dække eller omslutte med et klædningsstykke</v>
+      </c>
+      <c r="K23" t="str">
+        <v>shrouded</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Det ville være sværere med mama, men hun tog så mange sovepiller, at hun ville sove tungt, indhyllet i duften af sine jasmin- og geraniumparfumer.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N23" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O23" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
+        <v/>
+      </c>
+      <c r="AB23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gradvis" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB23"/>
+  <dimension ref="A1:AB24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2203,9 +2203,95 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>75dcfdca-1936-466f-a2b2-22a2a941a225</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C24" t="str">
+        <v>gradvis</v>
+      </c>
+      <c r="D24" t="str">
+        <v>gradvis</v>
+      </c>
+      <c r="E24" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v>- eller -t, -e</v>
+      </c>
+      <c r="H24" t="str">
+        <v>[ˈgʁɑðˌviˀs]</v>
+      </c>
+      <c r="I24" t="str">
+        <v>https://static.ordnet.dk/mp3/11018/11018445_1.mp3</v>
+      </c>
+      <c r="J24" t="str">
+        <v>som foregår lidt efter lidt eller trinvis</v>
+      </c>
+      <c r="K24" t="str">
+        <v>gradually</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Selvom hun gradvis havde skruet op for dosen af sovepiller, vågnede hun stadig grådkvalt midt om natten.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N24" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O24" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
+        <v/>
+      </c>
+      <c r="AA24" t="str">
+        <v/>
+      </c>
+      <c r="AB24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "skruet" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB24"/>
+  <dimension ref="A1:AB25"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2289,9 +2289,95 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>9cf7790a-5e18-4d37-8772-402bb9aa1e56</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C25" t="str">
+        <v>skruet</v>
+      </c>
+      <c r="D25" t="str">
+        <v>skrue</v>
+      </c>
+      <c r="E25" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H25" t="str">
+        <v>[ˈsgʁuːə]</v>
+      </c>
+      <c r="I25" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047030_1.mp3</v>
+      </c>
+      <c r="J25" t="str">
+        <v>dreje en skrue ind i eller ud af en genstand typisk ved hjælp af en skruetrækker</v>
+      </c>
+      <c r="K25" t="str">
+        <v>screwed</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Selvom hun gradvis havde skruet op for dosen af sovepiller, vågnede hun stadig grådkvalt midt om natten.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N25" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O25" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
+      <c r="W25" t="str">
+        <v/>
+      </c>
+      <c r="X25" t="str">
+        <v/>
+      </c>
+      <c r="Y25" t="str">
+        <v/>
+      </c>
+      <c r="Z25" t="str">
+        <v/>
+      </c>
+      <c r="AA25" t="str">
+        <v/>
+      </c>
+      <c r="AB25" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "grådkvalt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB25"/>
+  <dimension ref="A1:AB26"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2375,9 +2375,95 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>16f8262c-b71f-4b2d-9e4a-7dfff77141ff</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C26" t="str">
+        <v>grådkvalt</v>
+      </c>
+      <c r="D26" t="str">
+        <v>grådkvalt</v>
+      </c>
+      <c r="E26" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v>-, -e</v>
+      </c>
+      <c r="H26" t="str">
+        <v>[ˈgʁɔðˌkvæˀld]</v>
+      </c>
+      <c r="I26" t="str">
+        <v>https://static.ordnet.dk/mp3/11019/11019010_1.mp3</v>
+      </c>
+      <c r="J26" t="str">
+        <v>uklar og utydelig pga. gråd</v>
+      </c>
+      <c r="K26" t="str">
+        <v>choked with tears</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Selvom hun gradvis havde skruet op for dosen af sovepiller, vågnede hun stadig grådkvalt midt om natten.</v>
+      </c>
+      <c r="M26" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N26" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O26" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+      <c r="Z26" t="str">
+        <v/>
+      </c>
+      <c r="AA26" t="str">
+        <v/>
+      </c>
+      <c r="AB26" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "styrtede" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB26"/>
+  <dimension ref="A1:AB27"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2461,9 +2461,95 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>b924137c-0129-4efd-b8a1-c8e04e181e18</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C27" t="str">
+        <v>styrtede</v>
+      </c>
+      <c r="D27" t="str">
+        <v>styrte</v>
+      </c>
+      <c r="E27" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H27" t="str">
+        <v>[ˈsdyɐ̯də]</v>
+      </c>
+      <c r="I27" t="str">
+        <v>https://static.ordnet.dk/mp3/11051/11051088_1.mp3</v>
+      </c>
+      <c r="J27" t="str">
+        <v>pludseligt eller uheldigt vælte eller falde voldsomt fra oprejst stilling, fra en position højt oppe eller under hurtig bevægelse fremad</v>
+      </c>
+      <c r="K27" t="str">
+        <v>crashed</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Så styrtede jeg ind for at høre, hvad der var sket, men det eneste jeg kunne se gennem den halvåbne dør, var mama, der lå utrøstelig i papas favn, som en lille pige, der kom sig efter et forfærdeligt mareridt.</v>
+      </c>
+      <c r="M27" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N27" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O27" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
+      </c>
+      <c r="Z27" t="str">
+        <v/>
+      </c>
+      <c r="AA27" t="str">
+        <v/>
+      </c>
+      <c r="AB27" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "styrtede" in Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB27"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2493,7 +2493,7 @@
         <v>pludseligt eller uheldigt vælte eller falde voldsomt fra oprejst stilling, fra en position højt oppe eller under hurtig bevægelse fremad</v>
       </c>
       <c r="K27" t="str">
-        <v>crashed</v>
+        <v>rushed (in) /crashed</v>
       </c>
       <c r="L27" t="str">
         <v>Så styrtede jeg ind for at høre, hvad der var sket, men det eneste jeg kunne se gennem den halvåbne dør, var mama, der lå utrøstelig i papas favn, som en lille pige, der kom sig efter et forfærdeligt mareridt.</v>

</xml_diff>

<commit_message>
Add word "lå" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AB28"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2547,9 +2547,95 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>a62d3ee0-4eee-4c50-b1f1-ce1a02aa029b</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C28" t="str">
+        <v>lå</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v>-r, lå, -t</v>
+      </c>
+      <c r="H28" t="str">
+        <v>[ˈlegə]</v>
+      </c>
+      <c r="I28" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030434_1.mp3</v>
+      </c>
+      <c r="J28" t="str">
+        <v>befinde sig i en stilling hvor kroppen er vandret eller udstrakt og hviler på et underlag om menneske, dyr eller krop</v>
+      </c>
+      <c r="K28" t="str">
+        <v>lay</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Hannah Berlin, 1939 Jeg var knap tolv år gammel, da jeg besluttede mig for at slå mine forældre ihjel.</v>
+      </c>
+      <c r="M28" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N28" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O28" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+      <c r="V28" t="str">
+        <v/>
+      </c>
+      <c r="W28" t="str">
+        <v/>
+      </c>
+      <c r="X28" t="str">
+        <v/>
+      </c>
+      <c r="Y28" t="str">
+        <v/>
+      </c>
+      <c r="Z28" t="str">
+        <v/>
+      </c>
+      <c r="AA28" t="str">
+        <v/>
+      </c>
+      <c r="AB28" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "utrøstelig" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB28"/>
+  <dimension ref="A1:AB29"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2633,9 +2633,95 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>f5433505-0de6-4341-b5f0-2b418b8420db</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C29" t="str">
+        <v>utrøstelig</v>
+      </c>
+      <c r="D29" t="str">
+        <v>utrøstelig</v>
+      </c>
+      <c r="E29" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H29" t="str">
+        <v>[uˈtʁœsdəli]</v>
+      </c>
+      <c r="I29" t="str">
+        <v>https://static.ordnet.dk/mp3/12005/12005371_1.mp3</v>
+      </c>
+      <c r="J29" t="str">
+        <v>som det (næsten) ikke er muligt at trøste eller få i bedre humør</v>
+      </c>
+      <c r="K29" t="str">
+        <v>inconsolable</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Så styrtede jeg ind for at høre, hvad der var sket, men det eneste jeg kunne se gennem den halvåbne dør, var mama, der lå utrøstelig i papas favn, som en lille pige, der kom sig efter et forfærdeligt mareridt.</v>
+      </c>
+      <c r="M29" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N29" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O29" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v/>
+      </c>
+      <c r="X29" t="str">
+        <v/>
+      </c>
+      <c r="Y29" t="str">
+        <v/>
+      </c>
+      <c r="Z29" t="str">
+        <v/>
+      </c>
+      <c r="AA29" t="str">
+        <v/>
+      </c>
+      <c r="AB29" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "favn" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB29"/>
+  <dimension ref="A1:AB30"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2719,9 +2719,95 @@
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>d4740f9f-b684-4004-83a2-5e484fd21080</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C30" t="str">
+        <v>favn</v>
+      </c>
+      <c r="D30" t="str">
+        <v>favn</v>
+      </c>
+      <c r="E30" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F30" t="str">
+        <v>en</v>
+      </c>
+      <c r="G30" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H30" t="str">
+        <v>[ˈfɑwˀn]</v>
+      </c>
+      <c r="I30" t="str">
+        <v>https://static.ordnet.dk/mp3/11012/11012527_1.mp3</v>
+      </c>
+      <c r="J30" t="str">
+        <v>greb der dannes mellem en persons overkrop og dennes udbredte eller omsluttende arme</v>
+      </c>
+      <c r="K30" t="str">
+        <v>embrace</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Så styrtede jeg ind for at høre, hvad der var sket, men det eneste jeg kunne se gennem den halvåbne dør, var mama, der lå utrøstelig i papas favn, som en lille pige, der kom sig efter et forfærdeligt mareridt.</v>
+      </c>
+      <c r="M30" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N30" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O30" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+      <c r="T30" t="str">
+        <v/>
+      </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+      <c r="V30" t="str">
+        <v/>
+      </c>
+      <c r="W30" t="str">
+        <v/>
+      </c>
+      <c r="X30" t="str">
+        <v/>
+      </c>
+      <c r="Y30" t="str">
+        <v/>
+      </c>
+      <c r="Z30" t="str">
+        <v/>
+      </c>
+      <c r="AA30" t="str">
+        <v/>
+      </c>
+      <c r="AB30" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forfærdeligt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB30"/>
+  <dimension ref="A1:AB31"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2805,9 +2805,95 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>aee3a01f-e4f0-46d1-a1d4-89e22fb63d16</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C31" t="str">
+        <v>forfærdeligt</v>
+      </c>
+      <c r="D31" t="str">
+        <v>forfærdelig</v>
+      </c>
+      <c r="E31" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H31" t="str">
+        <v>[fʌˈfæɐ̯ˀdli]</v>
+      </c>
+      <c r="I31" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014510_1.mp3</v>
+      </c>
+      <c r="J31" t="str">
+        <v>som vækker stor forfærdelse; særdeles slem og ubehagelig</v>
+      </c>
+      <c r="K31" t="str">
+        <v>terrible</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Så styrtede jeg ind for at høre, hvad der var sket, men det eneste jeg kunne se gennem den halvåbne dør, var mama, der lå utrøstelig i papas favn, som en lille pige, der kom sig efter et forfærdeligt mareridt.</v>
+      </c>
+      <c r="M31" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N31" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O31" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
+        <v/>
+      </c>
+      <c r="T31" t="str">
+        <v/>
+      </c>
+      <c r="U31" t="str">
+        <v/>
+      </c>
+      <c r="V31" t="str">
+        <v/>
+      </c>
+      <c r="W31" t="str">
+        <v/>
+      </c>
+      <c r="X31" t="str">
+        <v/>
+      </c>
+      <c r="Y31" t="str">
+        <v/>
+      </c>
+      <c r="Z31" t="str">
+        <v/>
+      </c>
+      <c r="AA31" t="str">
+        <v/>
+      </c>
+      <c r="AB31" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "mareridt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB31"/>
+  <dimension ref="A1:AB32"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2891,9 +2891,95 @@
         <v/>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>38ca2e13-7bfc-4706-b756-b789ba12ade9</v>
+      </c>
+      <c r="B32" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C32" t="str">
+        <v>mareridt</v>
+      </c>
+      <c r="D32" t="str">
+        <v>mareridt</v>
+      </c>
+      <c r="E32" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F32" t="str">
+        <v>et</v>
+      </c>
+      <c r="G32" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H32" t="str">
+        <v>[ˈmɑːɑˌʁid]</v>
+      </c>
+      <c r="I32" t="str">
+        <v>https://static.ordnet.dk/mp3/11032/11032443_1.mp3</v>
+      </c>
+      <c r="J32" t="str">
+        <v>meget ubehagelig drøm der indeholder skræmmende eller forfærdelige indtryk og synsbilleder, ofte i en sådan grad at man sveder, får åndenød eller vågner af det</v>
+      </c>
+      <c r="K32" t="str">
+        <v>nightmare</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Så styrtede jeg ind for at høre, hvad der var sket, men det eneste jeg kunne se gennem den halvåbne dør, var mama, der lå utrøstelig i papas favn, som en lille pige, der kom sig efter et forfærdeligt mareridt.</v>
+      </c>
+      <c r="M32" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N32" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O32" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
+        <v/>
+      </c>
+      <c r="W32" t="str">
+        <v/>
+      </c>
+      <c r="X32" t="str">
+        <v/>
+      </c>
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
+        <v/>
+      </c>
+      <c r="AA32" t="str">
+        <v/>
+      </c>
+      <c r="AB32" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Bortset" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB32"/>
+  <dimension ref="A1:AB33"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2977,9 +2977,95 @@
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>5dffa7df-9745-4671-9468-138201e0e2aa</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Bortset</v>
+      </c>
+      <c r="D33" t="str">
+        <v>bortset</v>
+      </c>
+      <c r="E33" t="str">
+        <v>adverbium</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v>[-ˌseˀd]</v>
+      </c>
+      <c r="I33" t="str">
+        <v>https://static.ordnet.dk/mp3/11005/11005883_1.mp3</v>
+      </c>
+      <c r="J33" t="str">
+        <v>kun i udtrykket:</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Apart</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Bortset fra at for hende bestod mareridtet i at være vågen.</v>
+      </c>
+      <c r="M33" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N33" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O33" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
+      </c>
+      <c r="AA33" t="str">
+        <v/>
+      </c>
+      <c r="AB33" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bestod" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB33"/>
+  <dimension ref="A1:AB34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3063,9 +3063,95 @@
         <v/>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>4b3b5b1f-e370-4a72-a809-5929c1037b38</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C34" t="str">
+        <v>bestod</v>
+      </c>
+      <c r="D34" t="str">
+        <v>bestå</v>
+      </c>
+      <c r="E34" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v>-r, bestod, -et</v>
+      </c>
+      <c r="H34" t="str">
+        <v>[beˈsdɔˀ]</v>
+      </c>
+      <c r="I34" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004344_1.mp3</v>
+      </c>
+      <c r="J34" t="str">
+        <v>være lavet eller sammensat af; have som bestanddel eller væsentligt træk</v>
+      </c>
+      <c r="K34" t="str">
+        <v>passed</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Bortset fra at for hende bestod mareridtet i at være vågen.</v>
+      </c>
+      <c r="M34" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N34" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O34" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
+      </c>
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v/>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
+      </c>
+      <c r="AA34" t="str">
+        <v/>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "græd" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB34"/>
+  <dimension ref="A1:AB35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3149,9 +3149,95 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>f9ed6ee6-f008-4784-8399-f0894c729f31</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C35" t="str">
+        <v>græd</v>
+      </c>
+      <c r="D35" t="str">
+        <v>græde</v>
+      </c>
+      <c r="E35" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v>-r, græd, grædt</v>
+      </c>
+      <c r="H35" t="str">
+        <v>[ˈgʁaːðə]</v>
+      </c>
+      <c r="I35" t="str">
+        <v>https://static.ordnet.dk/mp3/11018/11018873_1.mp3</v>
+      </c>
+      <c r="J35" t="str">
+        <v>(spontant og ukontrolleret) lade tårer løbe fra øjnene som udtryk for en bestemt følelse, fx sorg, angst eller glæde, ofte samtidig med at man frembringer klagelyde, snapper efter vejret og snøfter</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Cry</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Ingen hørte længere, når jeg græd; det var der ingen, der tog sig af.</v>
+      </c>
+      <c r="M35" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N35" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O35" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v/>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
+        <v/>
+      </c>
+      <c r="AA35" t="str">
+        <v/>
+      </c>
+      <c r="AB35" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Ingen" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB35"/>
+  <dimension ref="A1:AB36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3235,9 +3235,95 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>c0d99d37-1a36-4a15-8793-714f792cabb9</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Ingen</v>
+      </c>
+      <c r="D36" t="str">
+        <v>ingen</v>
+      </c>
+      <c r="E36" t="str">
+        <v>pronomen</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v>intet, -</v>
+      </c>
+      <c r="H36" t="str">
+        <v>[ˈeŋən]</v>
+      </c>
+      <c r="I36" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023761_1.mp3</v>
+      </c>
+      <c r="J36" t="str">
+        <v>ikke en eneste; slet ikke nogen eller noget af det omtalte</v>
+      </c>
+      <c r="K36" t="str">
+        <v>No (one)</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Ingen hørte længere, når jeg græd; det var der ingen, der tog sig af.</v>
+      </c>
+      <c r="M36" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N36" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O36" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v/>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v/>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v/>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
+      </c>
+      <c r="AA36" t="str">
+        <v/>
+      </c>
+      <c r="AB36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Smerten" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB36"/>
+  <dimension ref="A1:AB37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3321,9 +3321,95 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>a72cbf20-890e-42e2-aa1f-039a5268b2b5</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Smerten</v>
+      </c>
+      <c r="D37" t="str">
+        <v>smerte</v>
+      </c>
+      <c r="E37" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F37" t="str">
+        <v>en</v>
+      </c>
+      <c r="G37" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H37" t="str">
+        <v>[ˈsmæɐ̯də]</v>
+      </c>
+      <c r="I37" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047986_1.mp3</v>
+      </c>
+      <c r="J37" t="str">
+        <v>stærkt ubehagelig sansefornemmelse fremkaldt af ydre vold eller en sygelig tilstand og oplevet som et pludseligt jag eller en vedvarende dunken eller murren i kroppen</v>
+      </c>
+      <c r="K37" t="str">
+        <v>The pain</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Smerten gnavede i hende.</v>
+      </c>
+      <c r="M37" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N37" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O37" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
+      <c r="S37" t="str">
+        <v/>
+      </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
+      <c r="U37" t="str">
+        <v/>
+      </c>
+      <c r="V37" t="str">
+        <v/>
+      </c>
+      <c r="W37" t="str">
+        <v/>
+      </c>
+      <c r="X37" t="str">
+        <v/>
+      </c>
+      <c r="Y37" t="str">
+        <v/>
+      </c>
+      <c r="Z37" t="str">
+        <v/>
+      </c>
+      <c r="AA37" t="str">
+        <v/>
+      </c>
+      <c r="AB37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gnavede" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB37"/>
+  <dimension ref="A1:AB38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3407,9 +3407,95 @@
         <v/>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>872ad8ba-3170-4538-83fe-c21858b6058d</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C38" t="str">
+        <v>gnavede</v>
+      </c>
+      <c r="D38" t="str">
+        <v>gnave</v>
+      </c>
+      <c r="E38" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H38" t="str">
+        <v>[ˈgnæːvə]</v>
+      </c>
+      <c r="I38" t="str">
+        <v>https://static.ordnet.dk/mp3/11018/11018279_1.mp3</v>
+      </c>
+      <c r="J38" t="str">
+        <v>bide med fortænderne gentagne gange og derved fjerne små stykker af noget spiseligt, et materiale el.lign. især om dyr</v>
+      </c>
+      <c r="K38" t="str">
+        <v>gnawed</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Smerten gnavede i hende.</v>
+      </c>
+      <c r="M38" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N38" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O38" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v/>
+      </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
+      <c r="W38" t="str">
+        <v/>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
+      <c r="Y38" t="str">
+        <v/>
+      </c>
+      <c r="Z38" t="str">
+        <v/>
+      </c>
+      <c r="AA38" t="str">
+        <v/>
+      </c>
+      <c r="AB38" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "stank" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB38"/>
+  <dimension ref="A1:AB39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3493,9 +3493,95 @@
         <v/>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>fd6cf519-3f56-476d-9997-fbd779ac6182</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C39" t="str">
+        <v>stank</v>
+      </c>
+      <c r="D39" t="str">
+        <v>stank</v>
+      </c>
+      <c r="E39" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F39" t="str">
+        <v>en</v>
+      </c>
+      <c r="G39" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H39" t="str">
+        <v>[ˈsdɑŋˀg]</v>
+      </c>
+      <c r="I39" t="str">
+        <v>https://static.ordnet.dk/mp3/11049/11049839_1.mp3</v>
+      </c>
+      <c r="J39" t="str">
+        <v>stærk, ubehagelig lugt</v>
+      </c>
+      <c r="K39" t="str">
+        <v>stink</v>
+      </c>
+      <c r="L39" t="str">
+        <v>dækket af smadret glas og den konstante stank af krudt, metal og røg bredte sig i gaderne, havde hun ligget og hulket hver nat.</v>
+      </c>
+      <c r="M39" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N39" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O39" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
+      <c r="AA39" t="str">
+        <v/>
+      </c>
+      <c r="AB39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB39"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "krudt" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB40"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3579,9 +3579,95 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>8c9e34e8-29de-41a3-b05e-d7e2d79dfd73</v>
+      </c>
+      <c r="B40" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C40" t="str">
+        <v>krudt</v>
+      </c>
+      <c r="D40" t="str">
+        <v>krudt</v>
+      </c>
+      <c r="E40" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F40" t="str">
+        <v>et</v>
+      </c>
+      <c r="G40" t="str">
+        <v>-et</v>
+      </c>
+      <c r="H40" t="str">
+        <v>[ˈkʁud]</v>
+      </c>
+      <c r="I40" t="str">
+        <v>https://static.ordnet.dk/mp3/11028/11028246_1.mp3</v>
+      </c>
+      <c r="J40" t="str">
+        <v>pulver som brænder eksplosivt uden lufttilførsel, og som bl.a. bruges i fyrværkeri og i skydevåben, hvor det ved eksplosionen driver projektilet fremad</v>
+      </c>
+      <c r="K40" t="str">
+        <v>powder</v>
+      </c>
+      <c r="L40" t="str">
+        <v>dækket af smadret glas og den konstante stank af krudt, metal og røg bredte sig i gaderne, havde hun ligget og hulket hver nat.</v>
+      </c>
+      <c r="M40" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N40" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O40" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v/>
+      </c>
+      <c r="X40" t="str">
+        <v/>
+      </c>
+      <c r="Y40" t="str">
+        <v/>
+      </c>
+      <c r="Z40" t="str">
+        <v/>
+      </c>
+      <c r="AA40" t="str">
+        <v/>
+      </c>
+      <c r="AB40" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bredte" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB40"/>
+  <dimension ref="A1:AB41"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3665,9 +3665,95 @@
         <v/>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>5eaac5bd-3c22-4ab5-92e8-d6215b5d9494</v>
+      </c>
+      <c r="B41" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C41" t="str">
+        <v>bredte</v>
+      </c>
+      <c r="D41" t="str">
+        <v>brede</v>
+      </c>
+      <c r="E41" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v>-r, bredte, bredt</v>
+      </c>
+      <c r="H41" t="str">
+        <v>[ˈbʁεːðə]</v>
+      </c>
+      <c r="I41" t="str">
+        <v>https://static.ordnet.dk/mp3/11006/11006085_1.mp3</v>
+      </c>
+      <c r="J41" t="str">
+        <v>sprede eller folde ud så overfladen dækker et større område</v>
+      </c>
+      <c r="K41" t="str">
+        <v>spread</v>
+      </c>
+      <c r="L41" t="str">
+        <v>dækket af smadret glas og den konstante stank af krudt, metal og røg bredte sig i gaderne, havde hun ligget og hulket hver nat.</v>
+      </c>
+      <c r="M41" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N41" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O41" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v/>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v/>
+      </c>
+      <c r="Y41" t="str">
+        <v/>
+      </c>
+      <c r="Z41" t="str">
+        <v/>
+      </c>
+      <c r="AA41" t="str">
+        <v/>
+      </c>
+      <c r="AB41" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ligget" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB41"/>
+  <dimension ref="A1:AB42"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3751,9 +3751,95 @@
         <v/>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>8f4aa8cf-20cf-494b-b2e5-21b000dad23f</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C42" t="str">
+        <v>ligget</v>
+      </c>
+      <c r="D42" t="str">
+        <v>ligge</v>
+      </c>
+      <c r="E42" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v>-r, lå, -t</v>
+      </c>
+      <c r="H42" t="str">
+        <v>[ˈlegə]</v>
+      </c>
+      <c r="I42" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030434_1.mp3</v>
+      </c>
+      <c r="J42" t="str">
+        <v>befinde sig i en stilling hvor kroppen er vandret eller udstrakt og hviler på et underlag om menneske, dyr eller krop</v>
+      </c>
+      <c r="K42" t="str">
+        <v>lying down</v>
+      </c>
+      <c r="L42" t="str">
+        <v>dækket af smadret glas og den konstante stank af krudt, metal og røg bredte sig i gaderne, havde hun ligget og hulket hver nat.</v>
+      </c>
+      <c r="M42" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N42" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O42" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v/>
+      </c>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v/>
+      </c>
+      <c r="Z42" t="str">
+        <v/>
+      </c>
+      <c r="AA42" t="str">
+        <v/>
+      </c>
+      <c r="AB42" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB42"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "hulket" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB42"/>
+  <dimension ref="A1:AB43"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3837,9 +3837,95 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>a3efef53-8d3d-4ead-adad-612c3eeaaaaf</v>
+      </c>
+      <c r="B43" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C43" t="str">
+        <v>hulket</v>
+      </c>
+      <c r="D43" t="str">
+        <v>hulk</v>
+      </c>
+      <c r="E43" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F43" t="str">
+        <v>et</v>
+      </c>
+      <c r="G43" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H43" t="str">
+        <v>[ˈhulˀg]</v>
+      </c>
+      <c r="I43" t="str">
+        <v>https://static.ordnet.dk/mp3/11021/11021562_1.mp3</v>
+      </c>
+      <c r="J43" t="str">
+        <v>hørlig snappen efter vejret under stærk sindsbevægelse, ofte under højlydt gråd; lyd der fremkommer derved</v>
+      </c>
+      <c r="K43" t="str">
+        <v>sobbed</v>
+      </c>
+      <c r="L43" t="str">
+        <v>dækket af smadret glas og den konstante stank af krudt, metal og røg bredte sig i gaderne, havde hun ligget og hulket hver nat.</v>
+      </c>
+      <c r="M43" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N43" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O43" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v/>
+      </c>
+      <c r="V43" t="str">
+        <v/>
+      </c>
+      <c r="W43" t="str">
+        <v/>
+      </c>
+      <c r="X43" t="str">
+        <v/>
+      </c>
+      <c r="Y43" t="str">
+        <v/>
+      </c>
+      <c r="Z43" t="str">
+        <v/>
+      </c>
+      <c r="AA43" t="str">
+        <v/>
+      </c>
+      <c r="AB43" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB43"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "smadret" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB43"/>
+  <dimension ref="A1:AB44"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3923,9 +3923,95 @@
         <v/>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>a17de7c4-96d3-4bdc-8670-6283bf490676</v>
+      </c>
+      <c r="B44" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C44" t="str">
+        <v>smadret</v>
+      </c>
+      <c r="D44" t="str">
+        <v>smadret</v>
+      </c>
+      <c r="E44" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v>-, smadrede</v>
+      </c>
+      <c r="H44" t="str">
+        <v>[ˈsmaðʁʌð]</v>
+      </c>
+      <c r="I44" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047919_1.mp3</v>
+      </c>
+      <c r="J44" t="str">
+        <v>se smadre</v>
+      </c>
+      <c r="K44" t="str">
+        <v>smashed</v>
+      </c>
+      <c r="L44" t="str">
+        <v>dækket af smadret glas og den konstante stank af krudt, metal og røg bredte sig i gaderne, havde hun ligget og hulket hver nat.</v>
+      </c>
+      <c r="M44" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N44" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O44" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v/>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v/>
+      </c>
+      <c r="V44" t="str">
+        <v/>
+      </c>
+      <c r="W44" t="str">
+        <v/>
+      </c>
+      <c r="X44" t="str">
+        <v/>
+      </c>
+      <c r="Y44" t="str">
+        <v/>
+      </c>
+      <c r="Z44" t="str">
+        <v/>
+      </c>
+      <c r="AA44" t="str">
+        <v/>
+      </c>
+      <c r="AB44" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB44"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forlade" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB44"/>
+  <dimension ref="A1:AB45"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4009,9 +4009,95 @@
         <v/>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>eb6ee03d-5421-43c9-bf55-c802b6a35054</v>
+      </c>
+      <c r="B45" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C45" t="str">
+        <v>forlade</v>
+      </c>
+      <c r="D45" t="str">
+        <v>forlade</v>
+      </c>
+      <c r="E45" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v>-r, forlod, forladt</v>
+      </c>
+      <c r="H45" t="str">
+        <v>[fʌˈlæˀðə]</v>
+      </c>
+      <c r="I45" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014710_1.mp3</v>
+      </c>
+      <c r="J45" t="str">
+        <v>gå, køre, sejle eller på anden måde bevæge sig væk fra et sted</v>
+      </c>
+      <c r="K45" t="str">
+        <v>leave</v>
+      </c>
+      <c r="L45" t="str">
+        <v>De besluttede, at vi skulle forlade det hjem, hvor jeg var født, og de forbød mig at gå hen i den skole, hvor ingen længere kunne lide mig.</v>
+      </c>
+      <c r="M45" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N45" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O45" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+      <c r="V45" t="str">
+        <v/>
+      </c>
+      <c r="W45" t="str">
+        <v/>
+      </c>
+      <c r="X45" t="str">
+        <v/>
+      </c>
+      <c r="Y45" t="str">
+        <v/>
+      </c>
+      <c r="Z45" t="str">
+        <v/>
+      </c>
+      <c r="AA45" t="str">
+        <v/>
+      </c>
+      <c r="AB45" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "tunge" in Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB45"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,7 +515,7 @@
         <v>muskelfyldt, aflangt og bevægeligt organ i mundhulen som bruges til at smage, slikke og (hos mennesket) frembringe tale med</v>
       </c>
       <c r="K4" t="str">
-        <v>tongue</v>
+        <v>heavy</v>
       </c>
       <c r="L4" t="str">
         <v>Jeg vidste altid hvornår, for papa lukkede de store tunge dobbeltvinduer og trak de tykke grønlige bronzefarvede gardiner for.</v>

</xml_diff>

<commit_message>
Add word "gardiner" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB45"/>
+  <dimension ref="A1:AB46"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4095,9 +4095,95 @@
         <v/>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>44c010e7-4c40-4c7b-bfd2-ddd078b76f46</v>
+      </c>
+      <c r="B46" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C46" t="str">
+        <v>gardiner</v>
+      </c>
+      <c r="D46" t="str">
+        <v>gardin</v>
+      </c>
+      <c r="E46" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F46" t="str">
+        <v>et</v>
+      </c>
+      <c r="G46" t="str">
+        <v>-et, -er, -erne</v>
+      </c>
+      <c r="H46" t="str">
+        <v>[gɑˈdiˀn]</v>
+      </c>
+      <c r="I46" t="str">
+        <v>https://static.ordnet.dk/mp3/11017/11017247_1.mp3</v>
+      </c>
+      <c r="J46" t="str">
+        <v>(dekorativt) stykke stof som indvendig i et rum hænger ned ved siden af eller foran et vindue for at skærme mod dagslys, for at forhindre at nogen kigger ind, eller som udsmykning ofte ophængt på en stang eller skinne således at det kan trækkes for e</v>
+      </c>
+      <c r="K46" t="str">
+        <v>Curtains</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Jeg vidste altid hvornår, for papa lukkede de store tunge dobbeltvinduer og trak de tykke grønlige bronzefarvede gardiner for.</v>
+      </c>
+      <c r="M46" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="N46" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="O46" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="P46" t="str">
+        <v/>
+      </c>
+      <c r="Q46" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+      <c r="S46" t="str">
+        <v/>
+      </c>
+      <c r="T46" t="str">
+        <v/>
+      </c>
+      <c r="U46" t="str">
+        <v/>
+      </c>
+      <c r="V46" t="str">
+        <v/>
+      </c>
+      <c r="W46" t="str">
+        <v/>
+      </c>
+      <c r="X46" t="str">
+        <v/>
+      </c>
+      <c r="Y46" t="str">
+        <v/>
+      </c>
+      <c r="Z46" t="str">
+        <v/>
+      </c>
+      <c r="AA46" t="str">
+        <v/>
+      </c>
+      <c r="AB46" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "bestod" in Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -195,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB46"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3095,7 +3095,7 @@
         <v>være lavet eller sammensat af; have som bestanddel eller væsentligt træk</v>
       </c>
       <c r="K34" t="str">
-        <v>passed</v>
+        <v>lie in/ consist of</v>
       </c>
       <c r="L34" t="str">
         <v>Bortset fra at for hende bestod mareridtet i at være vågen.</v>

</xml_diff>

<commit_message>
Add phrase "lige meget" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -4190,30 +4190,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4352,9 +4352,77 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>9aef9bb7-f445-413c-9dc0-86a16bc27333</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C3" t="str">
+        <v>lige meget</v>
+      </c>
+      <c r="D3" t="str">
+        <v>lige=just · meget=very</v>
+      </c>
+      <c r="E3" t="str">
+        <v>no matter</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Papa sagde til mig, at jeg var stærk, at jeg ville overleve, lige meget hvad der skete.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>| Biblioteket Sønderborg · Dentyskepige-4</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=13501465-62fa-43f6-b075-9b9388e402a1</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bidrage" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,36 +193,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB46"/>
+  <dimension ref="A1:AB47"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4181,9 +4181,95 @@
         <v/>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>e510b5f3-518e-4c8b-bde1-2ea7a53270c9</v>
+      </c>
+      <c r="B47" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="C47" t="str">
+        <v>bidrage</v>
+      </c>
+      <c r="D47" t="str">
+        <v>bidrage</v>
+      </c>
+      <c r="E47" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v>-r, bidrog (eller -de), -t</v>
+      </c>
+      <c r="H47" t="str">
+        <v>[ˈbiˌdʁɑˀwə]</v>
+      </c>
+      <c r="I47" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004596_1.mp3</v>
+      </c>
+      <c r="J47" t="str">
+        <v>medvirke (med arbejdsindsats, penge eller andet) til et fælles foretagende</v>
+      </c>
+      <c r="K47" t="str">
+        <v>contribute</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Internationale studerende kan bidrage med nyt perspektiv, solide kompetencer og kulturel forståelse i danske virksomheder 🌐 Men som ny i Danmark kan det være svært at vide, hvor man skal starte, når man gerne vil lan …</v>
+      </c>
+      <c r="M47" t="str">
+        <v>Feed | LinkedIn</v>
+      </c>
+      <c r="N47" t="str">
+        <v>https://www.linkedin.com/feed/</v>
+      </c>
+      <c r="O47" t="str">
+        <v>https://www.linkedin.com/feed/#:~:text=bidrage</v>
+      </c>
+      <c r="P47" t="str">
+        <v/>
+      </c>
+      <c r="Q47" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
+      <c r="S47" t="str">
+        <v/>
+      </c>
+      <c r="T47" t="str">
+        <v/>
+      </c>
+      <c r="U47" t="str">
+        <v/>
+      </c>
+      <c r="V47" t="str">
+        <v/>
+      </c>
+      <c r="W47" t="str">
+        <v/>
+      </c>
+      <c r="X47" t="str">
+        <v/>
+      </c>
+      <c r="Y47" t="str">
+        <v/>
+      </c>
+      <c r="Z47" t="str">
+        <v/>
+      </c>
+      <c r="AA47" t="str">
+        <v/>
+      </c>
+      <c r="AB47" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4192,28 +4278,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "nedbrud" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB47"/>
+  <dimension ref="A1:AB48"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4267,9 +4267,95 @@
         <v/>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>54c22739-f9be-41dc-962d-63934ab7759a</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="C48" t="str">
+        <v>nedbrud</v>
+      </c>
+      <c r="D48" t="str">
+        <v>nedbrud</v>
+      </c>
+      <c r="E48" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F48" t="str">
+        <v>et</v>
+      </c>
+      <c r="G48" t="str">
+        <v>-det, -, -dene</v>
+      </c>
+      <c r="H48" t="str">
+        <v>[ˈneðˌbʁuð]</v>
+      </c>
+      <c r="I48" t="str">
+        <v>https://static.ordnet.dk/mp3/11035/11035622_1.mp3</v>
+      </c>
+      <c r="J48" t="str">
+        <v>det at noget bryder ned eller bryder sammen</v>
+      </c>
+      <c r="K48" t="str">
+        <v>breakdown</v>
+      </c>
+      <c r="L48" t="str">
+        <v>En kvart milliard skal sikre 800.000 husstande mod strømnedbrud: »Det er især truslen fra fysiske angreb«</v>
+      </c>
+      <c r="M48" t="str">
+        <v>En kvart milliard skal sikre 800.000 husstande mod strømnedbrud: »Det er især truslen fra fysiske angreb« | Ingeniøren</v>
+      </c>
+      <c r="N48" t="str">
+        <v>https://ing.dk/artikel/en-kvart-milliard-skal-sikre-800000-husstande-mod-stroemnedbrud-det-er-isaer-truslen-fra-fysiske</v>
+      </c>
+      <c r="O48" t="str">
+        <v>https://ing.dk/artikel/en-kvart-milliard-skal-sikre-800000-husstande-mod-stroemnedbrud-det-er-isaer-truslen-fra-fysiske#:~:text=nedbrud</v>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
+      <c r="W48" t="str">
+        <v/>
+      </c>
+      <c r="X48" t="str">
+        <v/>
+      </c>
+      <c r="Y48" t="str">
+        <v/>
+      </c>
+      <c r="Z48" t="str">
+        <v/>
+      </c>
+      <c r="AA48" t="str">
+        <v/>
+      </c>
+      <c r="AB48" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: delete 1 in Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB48"/>
+  <dimension ref="A1:AB47"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4267,95 +4267,9 @@
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>54c22739-f9be-41dc-962d-63934ab7759a</v>
-      </c>
-      <c r="B48" t="str">
-        <v>2026-09-18</v>
-      </c>
-      <c r="C48" t="str">
-        <v>nedbrud</v>
-      </c>
-      <c r="D48" t="str">
-        <v>nedbrud</v>
-      </c>
-      <c r="E48" t="str">
-        <v>substantiv</v>
-      </c>
-      <c r="F48" t="str">
-        <v>et</v>
-      </c>
-      <c r="G48" t="str">
-        <v>-det, -, -dene</v>
-      </c>
-      <c r="H48" t="str">
-        <v>[ˈneðˌbʁuð]</v>
-      </c>
-      <c r="I48" t="str">
-        <v>https://static.ordnet.dk/mp3/11035/11035622_1.mp3</v>
-      </c>
-      <c r="J48" t="str">
-        <v>det at noget bryder ned eller bryder sammen</v>
-      </c>
-      <c r="K48" t="str">
-        <v>breakdown</v>
-      </c>
-      <c r="L48" t="str">
-        <v>En kvart milliard skal sikre 800.000 husstande mod strømnedbrud: »Det er især truslen fra fysiske angreb«</v>
-      </c>
-      <c r="M48" t="str">
-        <v>En kvart milliard skal sikre 800.000 husstande mod strømnedbrud: »Det er især truslen fra fysiske angreb« | Ingeniøren</v>
-      </c>
-      <c r="N48" t="str">
-        <v>https://ing.dk/artikel/en-kvart-milliard-skal-sikre-800000-husstande-mod-stroemnedbrud-det-er-isaer-truslen-fra-fysiske</v>
-      </c>
-      <c r="O48" t="str">
-        <v>https://ing.dk/artikel/en-kvart-milliard-skal-sikre-800000-husstande-mod-stroemnedbrud-det-er-isaer-truslen-fra-fysiske#:~:text=nedbrud</v>
-      </c>
-      <c r="P48" t="str">
-        <v/>
-      </c>
-      <c r="Q48" t="str">
-        <v>ok</v>
-      </c>
-      <c r="R48" t="str">
-        <v/>
-      </c>
-      <c r="S48" t="str">
-        <v/>
-      </c>
-      <c r="T48" t="str">
-        <v/>
-      </c>
-      <c r="U48" t="str">
-        <v/>
-      </c>
-      <c r="V48" t="str">
-        <v/>
-      </c>
-      <c r="W48" t="str">
-        <v/>
-      </c>
-      <c r="X48" t="str">
-        <v/>
-      </c>
-      <c r="Y48" t="str">
-        <v/>
-      </c>
-      <c r="Z48" t="str">
-        <v/>
-      </c>
-      <c r="AA48" t="str">
-        <v/>
-      </c>
-      <c r="AB48" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forhåbentlig" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB47"/>
+  <dimension ref="A1:AB48"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4267,9 +4267,95 @@
         <v/>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>5974aa41-7925-4231-9a67-2fa69172b310</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="C48" t="str">
+        <v>forhåbentlig</v>
+      </c>
+      <c r="D48" t="str">
+        <v>forhåbentlig</v>
+      </c>
+      <c r="E48" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H48" t="str">
+        <v>[fʌˈhɔˀbənli]</v>
+      </c>
+      <c r="I48" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014619_1.mp3</v>
+      </c>
+      <c r="J48" t="str">
+        <v>som man håber på vil blive resultatet</v>
+      </c>
+      <c r="K48" t="str">
+        <v>hopefully</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Næste uge kan blive en god uge… For både Grønland, Danmark og USA. Hvor lang tids usikkerhed forhåbentlig erstattes af en bindende aftale, der styrker sikkerheden i Ark</v>
+      </c>
+      <c r="M48" t="str">
+        <v>(3) Facebook</v>
+      </c>
+      <c r="N48" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O48" t="str">
+        <v>https://www.facebook.com/#:~:text=forh%C3%A5bentlig</v>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
+      <c r="W48" t="str">
+        <v/>
+      </c>
+      <c r="X48" t="str">
+        <v/>
+      </c>
+      <c r="Y48" t="str">
+        <v/>
+      </c>
+      <c r="Z48" t="str">
+        <v/>
+      </c>
+      <c r="AA48" t="str">
+        <v/>
+      </c>
+      <c r="AB48" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "erstattes" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB47"/>
+  <dimension ref="A1:AB48"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4267,9 +4267,95 @@
         <v/>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>109a0aad-5945-4497-8261-2d6c5bfa2530</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="C48" t="str">
+        <v>erstattes</v>
+      </c>
+      <c r="D48" t="str">
+        <v>erstatte</v>
+      </c>
+      <c r="E48" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H48" t="str">
+        <v>[æɐ̯ˈsdadə]</v>
+      </c>
+      <c r="I48" t="str">
+        <v>https://static.ordnet.dk/mp3/11011/11011757_1.mp3</v>
+      </c>
+      <c r="J48" t="str">
+        <v>sætte noget tilsvarende i stedet for noget som er tabt, forsvundet, ødelagt el.lign., eller som menes at være dårligere</v>
+      </c>
+      <c r="K48" t="str">
+        <v>be replaced</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Næste uge kan blive en god uge… For både Grønland, Danmark og USA. Hvor lang tids usikkerhed forhåbentlig erstattes af en bindende aftale, der styrker sikkerheden i Ark</v>
+      </c>
+      <c r="M48" t="str">
+        <v>(3) Facebook</v>
+      </c>
+      <c r="N48" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O48" t="str">
+        <v>https://www.facebook.com/#:~:text=erstattes</v>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
+      <c r="W48" t="str">
+        <v/>
+      </c>
+      <c r="X48" t="str">
+        <v/>
+      </c>
+      <c r="Y48" t="str">
+        <v/>
+      </c>
+      <c r="Z48" t="str">
+        <v/>
+      </c>
+      <c r="AA48" t="str">
+        <v/>
+      </c>
+      <c r="AB48" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bindende" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB48"/>
+  <dimension ref="A1:AB49"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4353,9 +4353,95 @@
         <v/>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>1682052c-f992-4d6f-97bb-599147db0a6d</v>
+      </c>
+      <c r="B49" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="C49" t="str">
+        <v>bindende</v>
+      </c>
+      <c r="D49" t="str">
+        <v>binde</v>
+      </c>
+      <c r="E49" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v>-r, bandt, bundet</v>
+      </c>
+      <c r="H49" t="str">
+        <v>[ˈbenə]</v>
+      </c>
+      <c r="I49" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004769_1.mp3</v>
+      </c>
+      <c r="J49" t="str">
+        <v>fastgøre eller samle med snor, reb el.lign. som man slår en knude på</v>
+      </c>
+      <c r="K49" t="str">
+        <v>Binding</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Næste uge kan blive en god uge… For både Grønland, Danmark og USA. Hvor lang tids usikkerhed forhåbentlig erstattes af en bindende aftale, der styrker sikkerheden i Ark</v>
+      </c>
+      <c r="M49" t="str">
+        <v>(3) Facebook</v>
+      </c>
+      <c r="N49" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O49" t="str">
+        <v>https://www.facebook.com/#:~:text=bindende</v>
+      </c>
+      <c r="P49" t="str">
+        <v/>
+      </c>
+      <c r="Q49" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R49" t="str">
+        <v/>
+      </c>
+      <c r="S49" t="str">
+        <v/>
+      </c>
+      <c r="T49" t="str">
+        <v/>
+      </c>
+      <c r="U49" t="str">
+        <v/>
+      </c>
+      <c r="V49" t="str">
+        <v/>
+      </c>
+      <c r="W49" t="str">
+        <v/>
+      </c>
+      <c r="X49" t="str">
+        <v/>
+      </c>
+      <c r="Y49" t="str">
+        <v/>
+      </c>
+      <c r="Z49" t="str">
+        <v/>
+      </c>
+      <c r="AA49" t="str">
+        <v/>
+      </c>
+      <c r="AB49" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "styrker" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AB50"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4439,9 +4439,95 @@
         <v/>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>479db00d-ac8f-4d61-acab-8d21a39d3204</v>
+      </c>
+      <c r="B50" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="C50" t="str">
+        <v>styrker</v>
+      </c>
+      <c r="D50" t="str">
+        <v>styrke</v>
+      </c>
+      <c r="E50" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F50" t="str">
+        <v>en</v>
+      </c>
+      <c r="G50" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H50" t="str">
+        <v>[ˈsdyɐ̯gə]</v>
+      </c>
+      <c r="I50" t="str">
+        <v>https://static.ordnet.dk/mp3/11051/11051073_1.mp3</v>
+      </c>
+      <c r="J50" t="str">
+        <v>fysisk eller psykisk kraft hos et menneske (eller et dyr)</v>
+      </c>
+      <c r="K50" t="str">
+        <v>Strengths</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Næste uge kan blive en god uge… For både Grønland, Danmark og USA. Hvor lang tids usikkerhed forhåbentlig erstattes af en bindende aftale, der styrker sikkerheden i Ark</v>
+      </c>
+      <c r="M50" t="str">
+        <v>(3) Facebook</v>
+      </c>
+      <c r="N50" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O50" t="str">
+        <v>https://www.facebook.com/#:~:text=styrker</v>
+      </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
+      <c r="Q50" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R50" t="str">
+        <v/>
+      </c>
+      <c r="S50" t="str">
+        <v/>
+      </c>
+      <c r="T50" t="str">
+        <v/>
+      </c>
+      <c r="U50" t="str">
+        <v/>
+      </c>
+      <c r="V50" t="str">
+        <v/>
+      </c>
+      <c r="W50" t="str">
+        <v/>
+      </c>
+      <c r="X50" t="str">
+        <v/>
+      </c>
+      <c r="Y50" t="str">
+        <v/>
+      </c>
+      <c r="Z50" t="str">
+        <v/>
+      </c>
+      <c r="AA50" t="str">
+        <v/>
+      </c>
+      <c r="AB50" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB50"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forandret" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB50"/>
+  <dimension ref="A1:AB51"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4525,9 +4525,95 @@
         <v/>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>f93e6623-051c-4adb-a379-ba2a0ab90c68</v>
+      </c>
+      <c r="B51" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="C51" t="str">
+        <v>forandret</v>
+      </c>
+      <c r="D51" t="str">
+        <v>forandre</v>
+      </c>
+      <c r="E51" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H51" t="str">
+        <v>[fʌˈɑnˀdʁʌ]</v>
+      </c>
+      <c r="I51" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014186_1.mp3</v>
+      </c>
+      <c r="J51" t="str">
+        <v>give en anden form, egenskab, karakter el.lign.</v>
+      </c>
+      <c r="K51" t="str">
+        <v>changed</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Det er vigtigt i en tid, hvor den sikkerhedspolitiske situation også i Arktis har forandret sig. See less</v>
+      </c>
+      <c r="M51" t="str">
+        <v>(3) Facebook</v>
+      </c>
+      <c r="N51" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O51" t="str">
+        <v>https://www.facebook.com/#:~:text=forandret</v>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R51" t="str">
+        <v/>
+      </c>
+      <c r="S51" t="str">
+        <v/>
+      </c>
+      <c r="T51" t="str">
+        <v/>
+      </c>
+      <c r="U51" t="str">
+        <v/>
+      </c>
+      <c r="V51" t="str">
+        <v/>
+      </c>
+      <c r="W51" t="str">
+        <v/>
+      </c>
+      <c r="X51" t="str">
+        <v/>
+      </c>
+      <c r="Y51" t="str">
+        <v/>
+      </c>
+      <c r="Z51" t="str">
+        <v/>
+      </c>
+      <c r="AA51" t="str">
+        <v/>
+      </c>
+      <c r="AB51" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB51"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "stikket" to Den Tyske Pige.xlsx
</commit_message>
<xml_diff>
--- a/sets/Den Tyske Pige.xlsx
+++ b/sets/Den Tyske Pige.xlsx
@@ -193,7 +193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB51"/>
+  <dimension ref="A1:AB52"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -4611,9 +4611,95 @@
         <v/>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>98bd79dc-4b61-4627-8a40-77b1134b991a</v>
+      </c>
+      <c r="B52" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="C52" t="str">
+        <v>stikket</v>
+      </c>
+      <c r="D52" t="str">
+        <v>stik</v>
+      </c>
+      <c r="E52" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F52" t="str">
+        <v>et</v>
+      </c>
+      <c r="G52" t="str">
+        <v>-ket, -, -kene</v>
+      </c>
+      <c r="H52" t="str">
+        <v>[ˈsdeg]</v>
+      </c>
+      <c r="I52" t="str">
+        <v>https://static.ordnet.dk/mp3/11050/11050243_1.mp3</v>
+      </c>
+      <c r="J52" t="str">
+        <v>det at bryde gennem en overflade med et spidst eller skarpt redskab, fx en kniv eller en kanyle</v>
+      </c>
+      <c r="K52" t="str">
+        <v>the plug</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Donglen kan findes til venstre under instrumentbrættet i OBD stikket (On-Board Diagnostics) Illustration: Mats Magnussen.</v>
+      </c>
+      <c r="M52" t="str">
+        <v>Nye biler får ekstra dongle til at overføre data: Sådan undgår du det | Ingeniøren</v>
+      </c>
+      <c r="N52" t="str">
+        <v>https://ing.dk/artikel/nye-biler-faar-ekstra-dongle-til-overfoere-data-saadan-undgaar-du-det</v>
+      </c>
+      <c r="O52" t="str">
+        <v>https://ing.dk/artikel/nye-biler-faar-ekstra-dongle-til-overfoere-data-saadan-undgaar-du-det#:~:text=stikket</v>
+      </c>
+      <c r="P52" t="str">
+        <v/>
+      </c>
+      <c r="Q52" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R52" t="str">
+        <v/>
+      </c>
+      <c r="S52" t="str">
+        <v/>
+      </c>
+      <c r="T52" t="str">
+        <v/>
+      </c>
+      <c r="U52" t="str">
+        <v/>
+      </c>
+      <c r="V52" t="str">
+        <v/>
+      </c>
+      <c r="W52" t="str">
+        <v/>
+      </c>
+      <c r="X52" t="str">
+        <v/>
+      </c>
+      <c r="Y52" t="str">
+        <v/>
+      </c>
+      <c r="Z52" t="str">
+        <v/>
+      </c>
+      <c r="AA52" t="str">
+        <v/>
+      </c>
+      <c r="AB52" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>